<commit_message>
the second half of the renaming sick
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset_NT_Dedup/H-2Kb_pcDelta_paired_convolved.xlsx
+++ b/Final_Figures_and_Sheets_Singleset_NT_Dedup/H-2Kb_pcDelta_paired_convolved.xlsx
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1.112582816131844e-10</v>
+        <v>1.075499501945527e-10</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>6.07939991752397e-09</v>
+        <v>5.946309688554705e-09</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>1.3480260892329e-07</v>
+        <v>1.329376652456161e-07</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>1.614465323019836e-06</v>
+        <v>1.599133162653992e-06</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>1.190196293453638e-05</v>
+        <v>1.181800642758516e-05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>5.874659421972416e-05</v>
+        <v>5.842475310810954e-05</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0002101632787898766</v>
+        <v>0.0002092195244275294</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>0.0005988767532098535</v>
+        <v>0.000596581426866526</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>0.001503436381077395</v>
+        <v>0.001498922753157812</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>0.003537736156043243</v>
+        <v>0.003530615464040578</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>0.007825825515108234</v>
+        <v>0.007814557584100363</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0160181866859882</v>
+        <v>0.01599569170969188</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>0.03022981008035846</v>
+        <v>0.03018345826399241</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>0.05269835018843168</v>
+        <v>0.05262004620267012</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="C41" t="n">
-        <v>0.08418528204839727</v>
+        <v>0.08408520888920649</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         <v>15</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1206271872793566</v>
+        <v>0.1205343160320225</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1508530649254565</v>
+        <v>0.1507964685416308</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1608866977072224</v>
+        <v>0.1608802142725789</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>18</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1443027362857559</v>
+        <v>0.144349896447004</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>19</v>
       </c>
       <c r="C46" t="n">
-        <v>0.1080255791893349</v>
+        <v>0.1081178499903559</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>20</v>
       </c>
       <c r="C47" t="n">
-        <v>0.06690504558650759</v>
+        <v>0.06701482402795741</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>0.03366642692861083</v>
+        <v>0.03375831440903575</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01328661980632581</v>
+        <v>0.01334339595423662</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>0.003841795317565789</v>
+        <v>0.003866232420913952</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0007247758707151072</v>
+        <v>0.0007322052018873087</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1353,7 +1353,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1371,7 +1371,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1389,7 +1389,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1407,7 +1407,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1425,7 +1425,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1443,7 +1443,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1461,7 +1461,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1479,7 +1479,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1497,7 +1497,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1515,7 +1515,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1533,7 +1533,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1551,7 +1551,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1569,7 +1569,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1587,7 +1587,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1605,7 +1605,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1623,7 +1623,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1641,7 +1641,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1659,7 +1659,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1677,7 +1677,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1695,7 +1695,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1713,7 +1713,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1731,7 +1731,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1749,7 +1749,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1767,7 +1767,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1785,7 +1785,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1803,7 +1803,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1821,7 +1821,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1839,7 +1839,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1857,7 +1857,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1875,7 +1875,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1893,7 +1893,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1911,7 +1911,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1929,7 +1929,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1947,7 +1947,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1965,7 +1965,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1983,7 +1983,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2001,7 +2001,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2019,7 +2019,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2037,7 +2037,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2055,7 +2055,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2073,7 +2073,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2091,7 +2091,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2109,7 +2109,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2127,7 +2127,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2145,7 +2145,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2163,7 +2163,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2181,7 +2181,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2199,7 +2199,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2217,7 +2217,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2235,7 +2235,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2253,7 +2253,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2271,7 +2271,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2289,7 +2289,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2307,7 +2307,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2325,7 +2325,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2343,7 +2343,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2361,7 +2361,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2379,7 +2379,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2397,7 +2397,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2415,7 +2415,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2433,7 +2433,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2451,7 +2451,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2469,7 +2469,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2487,7 +2487,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2505,7 +2505,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2523,7 +2523,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2541,7 +2541,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2559,7 +2559,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2577,7 +2577,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2595,7 +2595,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2613,7 +2613,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2631,7 +2631,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2649,7 +2649,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2667,7 +2667,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2685,7 +2685,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2703,7 +2703,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2721,7 +2721,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2739,7 +2739,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2757,7 +2757,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2775,7 +2775,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2793,7 +2793,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2811,7 +2811,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2829,7 +2829,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2847,7 +2847,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2865,7 +2865,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2883,7 +2883,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2901,7 +2901,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2919,7 +2919,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2937,7 +2937,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2955,7 +2955,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2973,7 +2973,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2991,7 +2991,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -3009,7 +3009,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -3027,7 +3027,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -3045,7 +3045,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -3063,7 +3063,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -3081,7 +3081,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -3099,7 +3099,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -3117,7 +3117,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -3135,7 +3135,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -3153,7 +3153,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -3171,7 +3171,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -3189,7 +3189,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -3207,7 +3207,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -3225,7 +3225,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -3243,7 +3243,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -3261,7 +3261,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -3279,7 +3279,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -3297,7 +3297,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -3315,7 +3315,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3333,7 +3333,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3351,7 +3351,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3369,7 +3369,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3387,7 +3387,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3405,7 +3405,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3423,7 +3423,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3441,7 +3441,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3459,7 +3459,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3477,7 +3477,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3495,7 +3495,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3513,7 +3513,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3531,7 +3531,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3549,7 +3549,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3567,7 +3567,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3585,7 +3585,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3603,7 +3603,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3621,7 +3621,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3639,7 +3639,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3657,7 +3657,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3675,7 +3675,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3693,7 +3693,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3711,7 +3711,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3729,7 +3729,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3747,7 +3747,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3765,7 +3765,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3783,7 +3783,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3801,7 +3801,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3819,7 +3819,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3837,7 +3837,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3855,7 +3855,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3873,7 +3873,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3891,7 +3891,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3909,7 +3909,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3927,7 +3927,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3945,7 +3945,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3963,7 +3963,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3981,7 +3981,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3999,7 +3999,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -4017,7 +4017,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -4035,7 +4035,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -4053,7 +4053,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -4071,7 +4071,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -4089,7 +4089,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -4107,7 +4107,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -4125,7 +4125,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -4143,7 +4143,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -4161,7 +4161,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -4179,7 +4179,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -4197,7 +4197,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -4215,7 +4215,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -4233,7 +4233,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -4251,7 +4251,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -4269,7 +4269,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -4287,7 +4287,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -4305,7 +4305,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -4323,7 +4323,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -4341,7 +4341,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -4359,7 +4359,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -4377,7 +4377,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -4395,7 +4395,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -4413,7 +4413,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -4431,7 +4431,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -4449,7 +4449,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4467,7 +4467,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4485,7 +4485,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4503,7 +4503,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4521,7 +4521,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4539,7 +4539,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4557,7 +4557,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4575,7 +4575,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4593,7 +4593,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4611,7 +4611,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4629,7 +4629,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4647,7 +4647,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4665,7 +4665,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4683,7 +4683,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4701,7 +4701,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4719,7 +4719,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4737,7 +4737,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4755,7 +4755,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4773,7 +4773,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4791,7 +4791,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4809,7 +4809,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4827,7 +4827,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4845,7 +4845,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4863,7 +4863,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4881,7 +4881,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4899,7 +4899,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4917,7 +4917,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4935,7 +4935,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4953,7 +4953,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4971,7 +4971,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4989,7 +4989,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -5007,7 +5007,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -5025,7 +5025,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -5043,7 +5043,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -5061,7 +5061,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -5079,7 +5079,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -5097,7 +5097,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -5115,7 +5115,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -5133,7 +5133,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -5151,7 +5151,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -5169,7 +5169,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -5187,7 +5187,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -5205,7 +5205,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -5223,7 +5223,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -5241,7 +5241,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -5259,7 +5259,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -5277,7 +5277,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -5295,7 +5295,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -5313,7 +5313,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -5331,7 +5331,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -5349,7 +5349,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -5367,7 +5367,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -5385,7 +5385,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -5403,7 +5403,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -5421,7 +5421,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -5439,7 +5439,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -5457,7 +5457,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -5475,7 +5475,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -5493,7 +5493,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -5511,7 +5511,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -5529,7 +5529,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -5547,7 +5547,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -5565,7 +5565,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5583,7 +5583,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5601,7 +5601,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5619,7 +5619,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5637,7 +5637,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5655,7 +5655,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5673,7 +5673,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5691,7 +5691,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5709,7 +5709,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5727,7 +5727,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5745,7 +5745,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5763,7 +5763,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5781,7 +5781,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5799,7 +5799,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5817,7 +5817,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5835,7 +5835,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5853,7 +5853,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5871,7 +5871,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5889,7 +5889,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5907,7 +5907,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5925,7 +5925,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5943,7 +5943,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5961,7 +5961,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5979,7 +5979,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5997,7 +5997,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -6015,7 +6015,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -6033,7 +6033,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -6051,7 +6051,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -6069,7 +6069,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -6087,7 +6087,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -6105,7 +6105,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -6123,7 +6123,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -6141,7 +6141,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -6159,7 +6159,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -6177,7 +6177,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -6195,7 +6195,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -6213,7 +6213,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -6231,7 +6231,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -6249,7 +6249,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -6267,7 +6267,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B325" t="n">
@@ -6285,7 +6285,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B326" t="n">

</xml_diff>